<commit_message>
Merge da branch do teste2-nelson
</commit_message>
<xml_diff>
--- a/consolidado_horarios.xlsx
+++ b/consolidado_horarios.xlsx
@@ -11,31 +11,31 @@
     <sheet name="Diêgo de Araujo Correia" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Erasmo da Silva Sà Junior" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Erick de Lima Mascarenhas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Hércules Porfirio" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Ian Tenório" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Jadiel Henrique" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="JOSE WENDER FERREIRA DUARTE" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="José Riquelme Teixeira da Silv" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="João Pedro" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="JULIA AZEVEDO PEREIRA" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Julia Gonçalves" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Kauã Lessa" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Laura Mainero" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Leandro Wanderley" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Hércules Porfirio de Jesus San" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Ian Carlos Cidreira Tenório" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Jadiel Henrique Calado Lino" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="José Riquelme Teixeira da Silv" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="José Wender Ferreira Duarte" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="João Pedro Simões da Silva Sou" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Julia Azevedo Pereira" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Julia Gonçalves dos Santos" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Kauã Lessa Lima dos Santos" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Laura Beatriz Lins Ramos Maine" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Leandro Wanderley Quintela Ten" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Ludson Lira de Almeida" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Luiz Bomfim" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Luiz Henrique Lima Leite" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Luiz Henrique Lima Leite" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Luiz Miguel de Melo Bomfim" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="Marcela Rocha Silva" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="Matheus Almeida Souza" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="Neilton Gabriel Goncalves" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="PEDRO ANDRE DA SILVA NETO" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Pedro André da Silva Neto" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="Pedro Henrique Feliciano da Si" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="PEDRO HENRIQUE OLIVEIRA NEVES" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Raul Alves" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Pedro Henrique Oliveira Neves" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Raul Alves do Nascimento" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="Victor Moura Amaral de Oliveir" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="WALTER SOARES COSTA NETO" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Wyvian Valença" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="YURI RAPHAEL MOTA DE ARAÚJO BA" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Walter Soares Costa Neto" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Wyvian Gabrielly Cavalcante VV" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Yuri Raphael Mota de Araújo Ba" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="Érico Almeida Bernardino" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
@@ -4412,7 +4412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4423,75 +4423,35 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Unnamed: 0</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Unnamed: 1</t>
+          <t>Seg</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Ter</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Seg</t>
+          <t>Qua</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Unnamed: 2</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Ter</t>
+          <t>Sex</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 3</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 4</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 5</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 6</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Qua</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Qui</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Sex</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 7</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Sab</t>
         </is>
@@ -4500,7 +4460,8 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>09:20 - 10:10</t>
+          <t>09:20 -
+10:10</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4513,44 +4474,37 @@
           <t>---</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>ECOM015</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ECOM019</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>ECOM015</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>COMP385</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+          <t>ECOM019</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10:10 - 11:00</t>
+          <t>10:10 -
+11:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4563,44 +4517,37 @@
           <t>---</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>ECOM015</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ECOM019</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>ECOM015</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>COMP385</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
+          <t>ECOM019</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>11:10 - 12:00</t>
+          <t>11:10 -
+12:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4610,38 +4557,30 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ECOM027</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ECOM015</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>ECOM015</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>ECOM027</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>---</t>
         </is>
@@ -4650,7 +4589,8 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>12:00 - 12:50</t>
+          <t>12:00 -
+12:50</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4660,38 +4600,30 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ECOM027</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ECOM015</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>ECOM015</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>ECOM027</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>---</t>
         </is>
@@ -4700,107 +4632,94 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>13:30 - 14:20</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
+          <t>13:30 -
+14:20</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ECOM020</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>COMP376</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+          <t>FALE0002</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ECOM020</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>COMP376</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>COMP377</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>14:20 - 15:10</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
+          <t>14:20 -
+15:10</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>ECOM020</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>COMP376</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
+          <t>FALE0002</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ECOM020</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>COMP376</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>COMP377</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>15:20 - 16:10</t>
+          <t>15:20 -
+16:10</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4810,47 +4729,40 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ECOM179</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>FALE0002</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>ECOM179</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>16:10 - 17:00</t>
+          <t>17:10 -
+18:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4860,42 +4772,77 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ECOM179</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>ECOM023</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>ECOM179</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
+          <t>ECOM023</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>18:00 -
+18:50</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ECOM023</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>ECOM023</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4908,7 +4855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4919,35 +4866,75 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed: 0</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Dom</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Seg</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 2</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Ter</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 3</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 4</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 5</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 6</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Qua</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Qui</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Sex</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 7</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Sab</t>
         </is>
@@ -4956,8 +4943,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>09:20 -
-10:10</t>
+          <t>09:20 - 10:10</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4970,37 +4956,44 @@
           <t>---</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>ECOM015</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>ECOM019</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>ECOM019</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>COMP385</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10:10 -
-11:00</t>
+          <t>10:10 - 11:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5013,37 +5006,44 @@
           <t>---</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>ECOM015</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>ECOM019</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>ECOM019</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>COMP385</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>11:10 -
-12:00</t>
+          <t>11:10 - 12:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5053,30 +5053,38 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+          <t>ECOM027</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
         <is>
           <t>ECOM015</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>ECOM027</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
         <is>
           <t>---</t>
         </is>
@@ -5085,8 +5093,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>12:00 -
-12:50</t>
+          <t>12:00 - 12:50</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -5096,30 +5103,38 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+          <t>ECOM027</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
         <is>
           <t>ECOM015</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>ECOM027</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
         <is>
           <t>---</t>
         </is>
@@ -5128,94 +5143,107 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>13:30 -
-14:20</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+          <t>13:30 - 14:20</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ECOM020</t>
+          <t>---</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>FALE0002</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>ECOM020</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+          <t>COMP376</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>COMP376</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>COMP377</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>14:20 -
-15:10</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+          <t>14:20 - 15:10</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ECOM020</t>
+          <t>---</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>FALE0002</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>ECOM020</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+          <t>COMP376</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>COMP376</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>COMP377</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>15:20 -
-16:10</t>
+          <t>15:20 - 16:10</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -5225,40 +5253,47 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>FALE0002</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+          <t>ECOM179</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ECOM179</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>17:10 -
-18:00</t>
+          <t>16:10 - 17:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -5268,77 +5303,42 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>ECOM023</t>
-        </is>
-      </c>
+          <t>ECOM179</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>ECOM023</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>18:00 -
-18:50</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>ECOM023</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>ECOM023</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ECOM179</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17868,6 +17868,502 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:P9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Horários</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Dom</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Seg</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Ter</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 1</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 2</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 3</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Qua</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 4</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Qui</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Sex</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 5</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Sab</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 6</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>09:20 - 10:10</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>COMP369</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>COMP369</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>10:10 - 11:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>COMP369</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>COMP369</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>11:10 - 12:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ECOM029</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ECOM029</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>12:00 - 12:50</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ECOM029</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ECOM029</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>13:30 - 14:20</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ECOM020</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>ECOM020</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>14:20 - 15:10</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ECOM020</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ECOM020</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>COMP383</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>15:20 - 16:10</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ECOM011</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>COMP389</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>ECOM011</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>COMP389</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>COMP383</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>16:10 - 17:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ECOM011</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>COMP389</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>ECOM011</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>COMP389</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:P34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -19573,500 +20069,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:P9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Horários</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 0</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Dom</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Seg</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Ter</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 1</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 2</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 3</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Qua</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 4</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Qui</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Sex</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 5</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Sab</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 6</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 7</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>09:20 - 10:10</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>COMP369</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>COMP369</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>10:10 - 11:00</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>COMP369</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>COMP369</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>11:10 - 12:00</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>ECOM029</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>ECOM029</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>12:00 - 12:50</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>ECOM029</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>ECOM029</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>13:30 - 14:20</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>ECOM020</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>ECOM020</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>14:20 - 15:10</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>ECOM020</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>ECOM020</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>COMP383</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>15:20 - 16:10</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>ECOM011</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>COMP389</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>ECOM011</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>COMP389</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>COMP383</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>16:10 - 17:00</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>ECOM011</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>COMP389</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>ECOM011</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>COMP389</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>